<commit_message>
modif employment series (SA)
</commit_message>
<xml_diff>
--- a/data/Data Germany.xlsx
+++ b/data/Data Germany.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timotheedangleterre/Desktop/ENSAE/Semestre 1/ESSD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85CDE3A6-D8DC-FF43-824E-BD45987BB555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC4E3D7B-7CB6-484B-AA0A-1C140E9CC25C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="1240" windowWidth="27640" windowHeight="16000" xr2:uid="{6454D7D1-463C-084D-BBBF-FAC872F6478C}"/>
+    <workbookView xWindow="720" yWindow="1020" windowWidth="27640" windowHeight="16000" activeTab="1" xr2:uid="{6454D7D1-463C-084D-BBBF-FAC872F6478C}"/>
   </bookViews>
   <sheets>
     <sheet name="Recettes" sheetId="1" r:id="rId1"/>
@@ -368,11 +368,11 @@
   <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="168" formatCode="#,##0.##########"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0"/>
-    <numFmt numFmtId="181" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.##########"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -383,12 +383,6 @@
     <font>
       <sz val="9"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
     <font>
@@ -480,13 +474,13 @@
     <xf numFmtId="3" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -497,7 +491,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1098,7 +1092,7 @@
         <v>57.1</v>
       </c>
       <c r="M2" s="13">
-        <v>39403</v>
+        <v>39775</v>
       </c>
       <c r="O2" s="8">
         <v>0.111848686020997</v>
@@ -1145,7 +1139,7 @@
         <v>57.4</v>
       </c>
       <c r="M3" s="13">
-        <v>39529</v>
+        <v>39856</v>
       </c>
       <c r="O3" s="8">
         <v>-5.9249511941494902E-3</v>
@@ -1192,7 +1186,7 @@
         <v>59</v>
       </c>
       <c r="M4" s="13">
-        <v>39650</v>
+        <v>39926</v>
       </c>
       <c r="O4" s="8">
         <v>-2.4606156303372401E-2</v>
@@ -1239,7 +1233,7 @@
         <v>57.9</v>
       </c>
       <c r="M5" s="13">
-        <v>39738</v>
+        <v>39952</v>
       </c>
       <c r="O5" s="8">
         <v>-4.20060243531672E-2</v>
@@ -1286,7 +1280,7 @@
         <v>58.4</v>
       </c>
       <c r="M6" s="13">
-        <v>39901</v>
+        <v>39981</v>
       </c>
       <c r="O6" s="8">
         <v>-3.01938662519508E-2</v>
@@ -1333,7 +1327,7 @@
         <v>60.6</v>
       </c>
       <c r="M7" s="13">
-        <v>40005</v>
+        <v>40022</v>
       </c>
       <c r="O7" s="8">
         <v>4.14806950729769E-2</v>
@@ -1380,7 +1374,7 @@
         <v>60.9</v>
       </c>
       <c r="M8" s="13">
-        <v>40063</v>
+        <v>40027</v>
       </c>
       <c r="O8" s="8">
         <v>3.62052223152887E-3</v>
@@ -1427,7 +1421,7 @@
         <v>60.9</v>
       </c>
       <c r="M9" s="13">
-        <v>40149</v>
+        <v>40044</v>
       </c>
       <c r="O9" s="8">
         <v>-5.9717048692890601E-2</v>
@@ -1474,7 +1468,7 @@
         <v>64.2</v>
       </c>
       <c r="M10" s="13">
-        <v>40352</v>
+        <v>40033</v>
       </c>
       <c r="O10" s="8">
         <v>4.0266131512263201E-2</v>
@@ -1521,7 +1515,7 @@
         <v>63.5</v>
       </c>
       <c r="M11" s="13">
-        <v>40352</v>
+        <v>40027</v>
       </c>
       <c r="O11" s="8">
         <v>-0.104947060075228</v>
@@ -1568,7 +1562,7 @@
         <v>64</v>
       </c>
       <c r="M12" s="13">
-        <v>40390</v>
+        <v>40030</v>
       </c>
       <c r="O12" s="8">
         <v>9.5705982046307998E-3</v>
@@ -1615,7 +1609,7 @@
         <v>63</v>
       </c>
       <c r="M13" s="13">
-        <v>40175</v>
+        <v>40037</v>
       </c>
       <c r="O13" s="8">
         <v>5.4671880647104501E-2</v>
@@ -1662,7 +1656,7 @@
         <v>62.4</v>
       </c>
       <c r="M14" s="13">
-        <v>39577</v>
+        <v>39944</v>
       </c>
       <c r="O14" s="8">
         <v>-9.0330191216073899E-2</v>
@@ -1709,7 +1703,7 @@
         <v>64.3</v>
       </c>
       <c r="M15" s="13">
-        <v>39605</v>
+        <v>39930</v>
       </c>
       <c r="O15" s="8">
         <v>-6.2869022181839498E-2</v>
@@ -1756,7 +1750,7 @@
         <v>64.2</v>
       </c>
       <c r="M16" s="13">
-        <v>39629</v>
+        <v>39912</v>
       </c>
       <c r="O16" s="8">
         <v>7.1891878087779304E-2</v>
@@ -1803,7 +1797,7 @@
         <v>65</v>
       </c>
       <c r="M17" s="13">
-        <v>39709</v>
+        <v>39922</v>
       </c>
       <c r="O17" s="8">
         <v>-2.2805739422519601E-2</v>
@@ -1850,7 +1844,7 @@
         <v>66.5</v>
       </c>
       <c r="M18" s="13">
-        <v>39854</v>
+        <v>39924</v>
       </c>
       <c r="O18" s="8">
         <v>-1.06521778957784E-2</v>
@@ -1897,7 +1891,7 @@
         <v>65.900000000000006</v>
       </c>
       <c r="M19" s="13">
-        <v>39856</v>
+        <v>39867</v>
       </c>
       <c r="O19" s="8">
         <v>-3.3089773619234798E-2</v>
@@ -1944,7 +1938,7 @@
         <v>64.5</v>
       </c>
       <c r="M20" s="13">
-        <v>39860</v>
+        <v>39827</v>
       </c>
       <c r="O20" s="8">
         <v>-0.12197162586308399</v>
@@ -1991,7 +1985,7 @@
         <v>64.2</v>
       </c>
       <c r="M21" s="13">
-        <v>39916</v>
+        <v>39816</v>
       </c>
       <c r="O21" s="8">
         <v>-0.18587246382334</v>
@@ -2038,7 +2032,7 @@
         <v>65.099999999999994</v>
       </c>
       <c r="M22" s="13">
-        <v>40096</v>
+        <v>39784</v>
       </c>
       <c r="O22" s="8">
         <v>5.6623235184378701E-2</v>
@@ -2085,7 +2079,7 @@
         <v>63</v>
       </c>
       <c r="M23" s="13">
-        <v>40127</v>
+        <v>39798</v>
       </c>
       <c r="O23" s="8">
         <v>9.0286114695754094E-2</v>
@@ -2132,7 +2126,7 @@
         <v>62</v>
       </c>
       <c r="M24" s="13">
-        <v>40177</v>
+        <v>39821</v>
       </c>
       <c r="O24" s="8">
         <v>3.35380732340873E-2</v>
@@ -2179,7 +2173,7 @@
         <v>61.4</v>
       </c>
       <c r="M25" s="13">
-        <v>39977</v>
+        <v>39836</v>
       </c>
       <c r="O25" s="8">
         <v>-1.02244204103847E-2</v>
@@ -2226,7 +2220,7 @@
         <v>62.7</v>
       </c>
       <c r="M26" s="13">
-        <v>39492</v>
+        <v>39859</v>
       </c>
       <c r="O26" s="8">
         <v>-1.35080164233585E-2</v>
@@ -2273,7 +2267,7 @@
         <v>63.1</v>
       </c>
       <c r="M27" s="13">
-        <v>39515</v>
+        <v>39842</v>
       </c>
       <c r="O27" s="8">
         <v>6.8673441743852606E-2</v>
@@ -2320,7 +2314,7 @@
         <v>64.2</v>
       </c>
       <c r="M28" s="13">
-        <v>39526</v>
+        <v>39817</v>
       </c>
       <c r="O28" s="8">
         <v>-6.8252795261562596E-2</v>
@@ -2367,7 +2361,7 @@
         <v>65.5</v>
       </c>
       <c r="M29" s="13">
-        <v>39612</v>
+        <v>39828</v>
       </c>
       <c r="O29" s="8">
         <v>-4.5223059505193702E-2</v>
@@ -2414,7 +2408,7 @@
         <v>64.7</v>
       </c>
       <c r="M30" s="13">
-        <v>39712</v>
+        <v>39776</v>
       </c>
       <c r="O30" s="8">
         <v>-9.4788086314228095E-2</v>
@@ -2461,7 +2455,7 @@
         <v>64.2</v>
       </c>
       <c r="M31" s="13">
-        <v>39683</v>
+        <v>39686</v>
       </c>
       <c r="O31" s="8">
         <v>-0.16926241416469001</v>
@@ -2508,7 +2502,7 @@
         <v>64.2</v>
       </c>
       <c r="M32" s="13">
-        <v>39711</v>
+        <v>39683</v>
       </c>
       <c r="O32" s="8">
         <v>3.4533721032712402E-3</v>
@@ -2555,7 +2549,7 @@
         <v>64.3</v>
       </c>
       <c r="M33" s="13">
-        <v>39699</v>
+        <v>39602</v>
       </c>
       <c r="O33" s="8">
         <v>-0.293326910897099</v>
@@ -2602,7 +2596,7 @@
         <v>65</v>
       </c>
       <c r="M34" s="13">
-        <v>39881</v>
+        <v>39568</v>
       </c>
       <c r="O34" s="8">
         <v>0.12980974771940601</v>
@@ -2649,7 +2643,7 @@
         <v>65.2</v>
       </c>
       <c r="M35" s="13">
-        <v>39860</v>
+        <v>39519</v>
       </c>
       <c r="O35" s="8">
         <v>5.1754347748044403E-2</v>
@@ -2696,7 +2690,7 @@
         <v>63.6</v>
       </c>
       <c r="M36" s="13">
-        <v>39823</v>
+        <v>39469</v>
       </c>
       <c r="O36" s="8">
         <v>-0.13789510203043201</v>
@@ -2743,7 +2737,7 @@
         <v>64</v>
       </c>
       <c r="M37" s="13">
-        <v>39576</v>
+        <v>39439</v>
       </c>
       <c r="O37" s="8">
         <v>-5.13545446787287E-2</v>
@@ -2790,7 +2784,7 @@
         <v>67</v>
       </c>
       <c r="M38" s="13">
-        <v>39024</v>
+        <v>39392</v>
       </c>
       <c r="O38" s="8">
         <v>-7.58756917913503E-2</v>
@@ -2837,7 +2831,7 @@
         <v>68.400000000000006</v>
       </c>
       <c r="M39" s="13">
-        <v>39048</v>
+        <v>39383</v>
       </c>
       <c r="O39" s="8">
         <v>-4.9570361160313298E-2</v>
@@ -2884,7 +2878,7 @@
         <v>68.900000000000006</v>
       </c>
       <c r="M40" s="13">
-        <v>39014</v>
+        <v>39308</v>
       </c>
       <c r="O40" s="8">
         <v>0.193737746804094</v>
@@ -2931,7 +2925,7 @@
         <v>66.7</v>
       </c>
       <c r="M41" s="13">
-        <v>38991</v>
+        <v>39207</v>
       </c>
       <c r="O41" s="8">
         <v>1.3718970746455599E-2</v>
@@ -2978,7 +2972,7 @@
         <v>65.5</v>
       </c>
       <c r="M42" s="13">
-        <v>39088</v>
+        <v>39150</v>
       </c>
       <c r="O42" s="8">
         <v>7.6739289513859901E-2</v>
@@ -3025,7 +3019,7 @@
         <v>65.900000000000006</v>
       </c>
       <c r="M43" s="13">
-        <v>39223</v>
+        <v>39218</v>
       </c>
       <c r="O43" s="8">
         <v>7.9726906607758594E-2</v>
@@ -3072,7 +3066,7 @@
         <v>66.099999999999994</v>
       </c>
       <c r="M44" s="13">
-        <v>39285</v>
+        <v>39258</v>
       </c>
       <c r="O44" s="8">
         <v>-9.4085555459777503E-4</v>
@@ -3119,7 +3113,7 @@
         <v>66.8</v>
       </c>
       <c r="M45" s="13">
-        <v>39296</v>
+        <v>39198</v>
       </c>
       <c r="O45" s="8">
         <v>-6.7608556684577395E-2</v>
@@ -3166,7 +3160,7 @@
         <v>66.5</v>
       </c>
       <c r="M46" s="13">
-        <v>39502</v>
+        <v>39186</v>
       </c>
       <c r="O46" s="8">
         <v>0.115627929501139</v>
@@ -3213,7 +3207,7 @@
         <v>66.599999999999994</v>
       </c>
       <c r="M47" s="13">
-        <v>39568</v>
+        <v>39215</v>
       </c>
       <c r="O47" s="8">
         <v>2.4308327639889899E-2</v>
@@ -3260,7 +3254,7 @@
         <v>66.3</v>
       </c>
       <c r="M48" s="13">
-        <v>39556</v>
+        <v>39202</v>
       </c>
       <c r="O48" s="8">
         <v>5.6870941869297198E-2</v>
@@ -3307,7 +3301,7 @@
         <v>66.2</v>
       </c>
       <c r="M49" s="13">
-        <v>39359</v>
+        <v>39225</v>
       </c>
       <c r="O49" s="8">
         <v>2.3291925425830601E-2</v>
@@ -3354,7 +3348,7 @@
         <v>66.900000000000006</v>
       </c>
       <c r="M50" s="13">
-        <v>38926</v>
+        <v>39299</v>
       </c>
       <c r="O50" s="8">
         <v>-1.0014046089356301E-2</v>
@@ -3401,7 +3395,7 @@
         <v>66.8</v>
       </c>
       <c r="M51" s="13">
-        <v>38969</v>
+        <v>39316</v>
       </c>
       <c r="O51" s="8">
         <v>-4.1012181651057099E-2</v>
@@ -3448,7 +3442,7 @@
         <v>67.400000000000006</v>
       </c>
       <c r="M52" s="13">
-        <v>39067</v>
+        <v>39370</v>
       </c>
       <c r="O52" s="8">
         <v>3.2778115786023E-2</v>
@@ -3495,7 +3489,7 @@
         <v>68.5</v>
       </c>
       <c r="M53" s="13">
-        <v>39213</v>
+        <v>39437</v>
       </c>
       <c r="O53" s="8">
         <v>-1.6138738075330401E-2</v>
@@ -3542,7 +3536,7 @@
         <v>70.3</v>
       </c>
       <c r="M54" s="13">
-        <v>39337</v>
+        <v>39400</v>
       </c>
       <c r="O54" s="8">
         <v>3.2939462694782803E-2</v>
@@ -3589,7 +3583,7 @@
         <v>69.2</v>
       </c>
       <c r="M55" s="13">
-        <v>39425</v>
+        <v>39410</v>
       </c>
       <c r="O55" s="8">
         <v>-3.9540417611966902E-2</v>
@@ -3636,7 +3630,7 @@
         <v>70</v>
       </c>
       <c r="M56" s="13">
-        <v>39412</v>
+        <v>39382</v>
       </c>
       <c r="O56" s="8">
         <v>-2.87489484783769E-2</v>
@@ -3683,7 +3677,7 @@
         <v>71.099999999999994</v>
       </c>
       <c r="M57" s="13">
-        <v>39480</v>
+        <v>39376</v>
       </c>
       <c r="O57" s="8">
         <v>2.80529988849079E-2</v>
@@ -3730,7 +3724,7 @@
         <v>70.599999999999994</v>
       </c>
       <c r="M58" s="13">
-        <v>39709</v>
+        <v>39386</v>
       </c>
       <c r="O58" s="8">
         <v>1.7152798504905999E-2</v>
@@ -3777,7 +3771,7 @@
         <v>72.900000000000006</v>
       </c>
       <c r="M59" s="13">
-        <v>39733</v>
+        <v>39369</v>
       </c>
       <c r="O59" s="8">
         <v>4.1001260062236297E-2</v>
@@ -3824,7 +3818,7 @@
         <v>71</v>
       </c>
       <c r="M60" s="13">
-        <v>39717</v>
+        <v>39361</v>
       </c>
       <c r="O60" s="8">
         <v>3.10401525621966E-2</v>
@@ -3871,7 +3865,7 @@
         <v>69.3</v>
       </c>
       <c r="M61" s="13">
-        <v>39454</v>
+        <v>39325</v>
       </c>
       <c r="O61" s="8">
         <v>-2.8903549950776202E-4</v>
@@ -3918,7 +3912,7 @@
         <v>70.5</v>
       </c>
       <c r="M62" s="13">
-        <v>38899</v>
+        <v>39274</v>
       </c>
       <c r="O62" s="8">
         <v>2.22290045964222E-2</v>
@@ -3965,7 +3959,7 @@
         <v>71.099999999999994</v>
       </c>
       <c r="M63" s="13">
-        <v>38914</v>
+        <v>39274</v>
       </c>
       <c r="O63" s="8">
         <v>-3.95485320812128E-4</v>
@@ -4012,7 +4006,7 @@
         <v>73.099999999999994</v>
       </c>
       <c r="M64" s="13">
-        <v>38932</v>
+        <v>39239</v>
       </c>
       <c r="O64" s="8">
         <v>-3.8424616894092302E-2</v>
@@ -4059,7 +4053,7 @@
         <v>74.7</v>
       </c>
       <c r="M65" s="13">
-        <v>39003</v>
+        <v>39226</v>
       </c>
       <c r="O65" s="8">
         <v>6.3821551296939602E-2</v>
@@ -4106,7 +4100,7 @@
         <v>74.5</v>
       </c>
       <c r="M66" s="13">
-        <v>39168</v>
+        <v>39232</v>
       </c>
       <c r="O66" s="8">
         <v>2.7779205722774598E-2</v>
@@ -4153,7 +4147,7 @@
         <v>76.2</v>
       </c>
       <c r="M67" s="13">
-        <v>39295</v>
+        <v>39274</v>
       </c>
       <c r="O67" s="8">
         <v>6.3407109683772903E-2</v>
@@ -4200,7 +4194,7 @@
         <v>78.099999999999994</v>
       </c>
       <c r="M68" s="13">
-        <v>39308</v>
+        <v>39271</v>
       </c>
       <c r="O68" s="8">
         <v>-1.16940295186438E-2</v>
@@ -4247,7 +4241,7 @@
         <v>79.2</v>
       </c>
       <c r="M69" s="13">
-        <v>39446</v>
+        <v>39339</v>
       </c>
       <c r="O69" s="8">
         <v>4.3440960416413398E-2</v>
@@ -4294,7 +4288,7 @@
         <v>81.8</v>
       </c>
       <c r="M70" s="13">
-        <v>39722</v>
+        <v>39397</v>
       </c>
       <c r="O70" s="8">
         <v>-2.30729380706549E-2</v>
@@ -4341,7 +4335,7 @@
         <v>82.1</v>
       </c>
       <c r="M71" s="13">
-        <v>39781</v>
+        <v>39413</v>
       </c>
       <c r="O71" s="8">
         <v>5.2238276234790597E-2</v>
@@ -4388,7 +4382,7 @@
         <v>79.3</v>
       </c>
       <c r="M72" s="13">
-        <v>39810</v>
+        <v>39455</v>
       </c>
       <c r="O72" s="8">
         <v>4.05388013129322E-2</v>
@@ -4435,7 +4429,7 @@
         <v>79.3</v>
       </c>
       <c r="M73" s="13">
-        <v>39588</v>
+        <v>39464</v>
       </c>
       <c r="O73" s="8">
         <v>4.7993384031359602E-2</v>
@@ -4482,7 +4476,7 @@
         <v>81.400000000000006</v>
       </c>
       <c r="M74" s="13">
-        <v>38906</v>
+        <v>39282</v>
       </c>
       <c r="O74" s="8">
         <v>2.12541772824348E-2</v>
@@ -4529,7 +4523,7 @@
         <v>81.5</v>
       </c>
       <c r="M75" s="13">
-        <v>38933</v>
+        <v>39298</v>
       </c>
       <c r="O75" s="8">
         <v>2.9585408250438799E-2</v>
@@ -4576,7 +4570,7 @@
         <v>81.7</v>
       </c>
       <c r="M76" s="13">
-        <v>39002</v>
+        <v>39313</v>
       </c>
       <c r="O76" s="8">
         <v>6.6461275641351803E-3</v>
@@ -4623,7 +4617,7 @@
         <v>84.2</v>
       </c>
       <c r="M77" s="13">
-        <v>39188</v>
+        <v>39406</v>
       </c>
       <c r="O77" s="8">
         <v>-5.4193734252946199E-2</v>
@@ -4670,7 +4664,7 @@
         <v>84.6</v>
       </c>
       <c r="M78" s="13">
-        <v>39475</v>
+        <v>39539</v>
       </c>
       <c r="O78" s="8">
         <v>-1.6789142560789099E-3</v>
@@ -4717,7 +4711,7 @@
         <v>85.2</v>
       </c>
       <c r="M79" s="13">
-        <v>39666</v>
+        <v>39646</v>
       </c>
       <c r="O79" s="8">
         <v>-2.3577839243316099E-4</v>
@@ -4764,7 +4758,7 @@
         <v>86</v>
       </c>
       <c r="M80" s="13">
-        <v>39748</v>
+        <v>39707</v>
       </c>
       <c r="O80" s="8">
         <v>3.0778150659468699E-2</v>
@@ -4811,7 +4805,7 @@
         <v>85.5</v>
       </c>
       <c r="M81" s="13">
-        <v>39847</v>
+        <v>39737</v>
       </c>
       <c r="O81" s="8">
         <v>2.4404696572020199E-2</v>
@@ -4858,7 +4852,7 @@
         <v>82.4</v>
       </c>
       <c r="M82" s="13">
-        <v>40080</v>
+        <v>39754</v>
       </c>
       <c r="O82" s="8">
         <v>4.3123189912208197E-2</v>
@@ -4905,7 +4899,7 @@
         <v>82</v>
       </c>
       <c r="M83" s="13">
-        <v>40144</v>
+        <v>39772</v>
       </c>
       <c r="O83" s="8">
         <v>6.4032128136766201E-3</v>
@@ -4952,7 +4946,7 @@
         <v>81.5</v>
       </c>
       <c r="M84" s="13">
-        <v>40226</v>
+        <v>39874</v>
       </c>
       <c r="O84" s="8">
         <v>4.4595570244412699E-2</v>
@@ -4999,7 +4993,7 @@
         <v>81.5</v>
       </c>
       <c r="M85" s="13">
-        <v>40078</v>
+        <v>39959</v>
       </c>
       <c r="O85" s="8">
         <v>2.8716976130818101E-2</v>
@@ -5046,7 +5040,7 @@
         <v>82.6</v>
       </c>
       <c r="M86" s="13">
-        <v>39652</v>
+        <v>40032</v>
       </c>
       <c r="O86" s="8">
         <v>-1.0910493683644201E-2</v>
@@ -5093,7 +5087,7 @@
         <v>83.3</v>
       </c>
       <c r="M87" s="13">
-        <v>39703</v>
+        <v>40077</v>
       </c>
       <c r="O87" s="8">
         <v>2.9577111641844001E-2</v>
@@ -5140,7 +5134,7 @@
         <v>84.6</v>
       </c>
       <c r="M88" s="13">
-        <v>39799</v>
+        <v>40115</v>
       </c>
       <c r="O88" s="8">
         <v>6.8691491180905104E-2</v>
@@ -5187,7 +5181,7 @@
         <v>85.7</v>
       </c>
       <c r="M89" s="13">
-        <v>39981</v>
+        <v>40189</v>
       </c>
       <c r="O89" s="8">
         <v>6.2035674360270597E-2</v>
@@ -5234,7 +5228,7 @@
         <v>86.3</v>
       </c>
       <c r="M90" s="13">
-        <v>40168</v>
+        <v>40227</v>
       </c>
       <c r="O90" s="8">
         <v>1.5642480139463899E-2</v>
@@ -5281,7 +5275,7 @@
         <v>86.5</v>
       </c>
       <c r="M91" s="13">
-        <v>40261</v>
+        <v>40244</v>
       </c>
       <c r="O91" s="8">
         <v>-5.4296858645066899E-2</v>
@@ -5328,7 +5322,7 @@
         <v>87.3</v>
       </c>
       <c r="M92" s="13">
-        <v>40352</v>
+        <v>40308</v>
       </c>
       <c r="O92" s="8">
         <v>7.0987927379011504E-3</v>
@@ -5375,7 +5369,7 @@
         <v>86.2</v>
       </c>
       <c r="M93" s="13">
-        <v>40463</v>
+        <v>40354</v>
       </c>
       <c r="O93" s="8">
         <v>2.8820634673508001E-2</v>
@@ -5422,7 +5416,7 @@
         <v>87.3</v>
       </c>
       <c r="M94" s="13">
-        <v>40694</v>
+        <v>40369</v>
       </c>
       <c r="O94" s="8">
         <v>1.98625169456275E-2</v>
@@ -5469,7 +5463,7 @@
         <v>87.1</v>
       </c>
       <c r="M95" s="13">
-        <v>40820</v>
+        <v>40452</v>
       </c>
       <c r="O95" s="8">
         <v>-1.8717050656217499E-2</v>
@@ -5516,7 +5510,7 @@
         <v>90.5</v>
       </c>
       <c r="M96" s="13">
-        <v>40843</v>
+        <v>40497</v>
       </c>
       <c r="O96" s="8">
         <v>2.4697174735417E-2</v>
@@ -5563,7 +5557,7 @@
         <v>88.5</v>
       </c>
       <c r="M97" s="13">
-        <v>40634</v>
+        <v>40519</v>
       </c>
       <c r="O97" s="8">
         <v>-0.16331721706246699</v>
@@ -5610,7 +5604,7 @@
         <v>90.4</v>
       </c>
       <c r="M98" s="13">
-        <v>40337</v>
+        <v>40715</v>
       </c>
       <c r="O98" s="8">
         <v>-1.52386819990173E-2</v>
@@ -5657,7 +5651,7 @@
         <v>90.8</v>
       </c>
       <c r="M99" s="13">
-        <v>40388</v>
+        <v>40762</v>
       </c>
       <c r="O99" s="8">
         <v>-3.2097622823616903E-2</v>
@@ -5704,7 +5698,7 @@
         <v>92.9</v>
       </c>
       <c r="M100" s="13">
-        <v>40465</v>
+        <v>40783</v>
       </c>
       <c r="O100" s="8">
         <v>6.14040464165004E-2</v>
@@ -5751,7 +5745,7 @@
         <v>93.7</v>
       </c>
       <c r="M101" s="13">
-        <v>40601</v>
+        <v>40795</v>
       </c>
       <c r="O101" s="8">
         <v>2.10707389491969E-2</v>
@@ -5798,7 +5792,7 @@
         <v>96.9</v>
       </c>
       <c r="M102" s="13">
-        <v>40743</v>
+        <v>40794</v>
       </c>
       <c r="O102" s="8">
         <v>-0.100486200815029</v>
@@ -5845,7 +5839,7 @@
         <v>98.7</v>
       </c>
       <c r="M103" s="13">
-        <v>40822</v>
+        <v>40807</v>
       </c>
       <c r="O103" s="8">
         <v>9.4962420404005599E-3</v>
@@ -5892,7 +5886,7 @@
         <v>100.1</v>
       </c>
       <c r="M104" s="13">
-        <v>40914</v>
+        <v>40872</v>
       </c>
       <c r="O104" s="8">
         <v>-8.8763372832740793E-3</v>
@@ -5939,7 +5933,7 @@
         <v>97.1</v>
       </c>
       <c r="M105" s="13">
-        <v>40978</v>
+        <v>40872</v>
       </c>
       <c r="O105" s="8">
         <v>-9.6584333056723495E-2</v>
@@ -5986,7 +5980,7 @@
         <v>97.7</v>
       </c>
       <c r="M106" s="13">
-        <v>41246</v>
+        <v>40924</v>
       </c>
       <c r="O106" s="8">
         <v>-0.15616288908964299</v>
@@ -6033,7 +6027,7 @@
         <v>95.4</v>
       </c>
       <c r="M107" s="13">
-        <v>41338</v>
+        <v>40977</v>
       </c>
       <c r="O107" s="8">
         <v>-6.5989918842177503E-2</v>
@@ -6080,7 +6074,7 @@
         <v>91.6</v>
       </c>
       <c r="M108" s="13">
-        <v>41303</v>
+        <v>40968</v>
       </c>
       <c r="O108" s="8">
         <v>2.9699566303380099E-2</v>
@@ -6127,7 +6121,7 @@
         <v>87.8</v>
       </c>
       <c r="M109" s="13">
-        <v>41079</v>
+        <v>40969</v>
       </c>
       <c r="O109" s="8">
         <v>-0.103244589896516</v>
@@ -6174,7 +6168,7 @@
         <v>89.7</v>
       </c>
       <c r="M110" s="13">
-        <v>40644</v>
+        <v>41013</v>
       </c>
       <c r="O110" s="8">
         <v>-0.121048265599494</v>
@@ -6221,7 +6215,7 @@
         <v>89.7</v>
       </c>
       <c r="M111" s="13">
-        <v>40664</v>
+        <v>41035</v>
       </c>
       <c r="O111" s="8">
         <v>6.0817129044151499E-2</v>
@@ -6268,7 +6262,7 @@
         <v>88.7</v>
       </c>
       <c r="M112" s="13">
-        <v>40675</v>
+        <v>40989</v>
       </c>
       <c r="O112" s="8">
         <v>0.154968057772958</v>
@@ -6315,7 +6309,7 @@
         <v>88.8</v>
       </c>
       <c r="M113" s="13">
-        <v>40783</v>
+        <v>40959</v>
       </c>
       <c r="O113" s="8">
         <v>3.53002385304464E-2</v>
@@ -6362,7 +6356,7 @@
         <v>89.3</v>
       </c>
       <c r="M114" s="13">
-        <v>40854</v>
+        <v>40894</v>
       </c>
       <c r="O114" s="8">
         <v>-2.7116945463070901E-2</v>
@@ -6409,7 +6403,7 @@
         <v>91</v>
       </c>
       <c r="M115" s="13">
-        <v>40863</v>
+        <v>40845</v>
       </c>
       <c r="O115" s="8">
         <v>0.103338355889289</v>
@@ -6456,7 +6450,7 @@
         <v>88.7</v>
       </c>
       <c r="M116" s="13">
-        <v>40870</v>
+        <v>40831</v>
       </c>
       <c r="O116" s="8">
         <v>2.4540046666183798E-2</v>
@@ -6503,7 +6497,7 @@
         <v>90.4</v>
       </c>
       <c r="M117" s="13">
-        <v>40941</v>
+        <v>40840</v>
       </c>
       <c r="O117" s="8">
         <v>3.7806053492298403E-2</v>
@@ -6550,7 +6544,7 @@
         <v>89</v>
       </c>
       <c r="M118" s="13">
-        <v>41174</v>
+        <v>40865</v>
       </c>
       <c r="O118" s="8">
         <v>-4.6933298011303699E-2</v>
@@ -6597,7 +6591,7 @@
         <v>88.8</v>
       </c>
       <c r="M119" s="13">
-        <v>41194</v>
+        <v>40849</v>
       </c>
       <c r="O119" s="8">
         <v>3.8224371112022502E-2</v>
@@ -6644,7 +6638,7 @@
         <v>89.3</v>
       </c>
       <c r="M120" s="13">
-        <v>41176</v>
+        <v>40855</v>
       </c>
       <c r="O120" s="8">
         <v>5.7249352097251502E-2</v>
@@ -6691,7 +6685,7 @@
         <v>88.6</v>
       </c>
       <c r="M121" s="13">
-        <v>40999</v>
+        <v>40898</v>
       </c>
       <c r="O121" s="8">
         <v>-6.0304192571880598E-2</v>
@@ -6738,7 +6732,7 @@
         <v>90.6</v>
       </c>
       <c r="M122" s="13">
-        <v>40524</v>
+        <v>40881</v>
       </c>
       <c r="O122" s="8">
         <v>-1.8434640166748999E-3</v>
@@ -6785,7 +6779,7 @@
         <v>89.8</v>
       </c>
       <c r="M123" s="13">
-        <v>40527</v>
+        <v>40888</v>
       </c>
       <c r="O123" s="8">
         <v>9.4537566370185303E-2</v>
@@ -6832,7 +6826,7 @@
         <v>92.2</v>
       </c>
       <c r="M124" s="13">
-        <v>40640</v>
+        <v>40948</v>
       </c>
       <c r="O124" s="8">
         <v>-2.90491639881196E-3</v>
@@ -6879,7 +6873,7 @@
         <v>93.4</v>
       </c>
       <c r="M125" s="13">
-        <v>40852</v>
+        <v>41014</v>
       </c>
       <c r="O125" s="8">
         <v>-2.8327462453287201E-2</v>
@@ -6926,7 +6920,7 @@
         <v>93.6</v>
       </c>
       <c r="M126" s="13">
-        <v>41030</v>
+        <v>41058</v>
       </c>
       <c r="O126" s="8">
         <v>1.99489750576376E-4</v>
@@ -6973,7 +6967,7 @@
         <v>93.5</v>
       </c>
       <c r="M127" s="13">
-        <v>41130</v>
+        <v>41106</v>
       </c>
       <c r="O127" s="8">
         <v>3.01257507613002E-2</v>
@@ -7020,7 +7014,7 @@
         <v>92.8</v>
       </c>
       <c r="M128" s="13">
-        <v>41160</v>
+        <v>41122</v>
       </c>
       <c r="O128" s="8">
         <v>-3.6904127581514998E-2</v>
@@ -7067,7 +7061,7 @@
         <v>92.6</v>
       </c>
       <c r="M129" s="13">
-        <v>41265</v>
+        <v>41168</v>
       </c>
       <c r="O129" s="8">
         <v>5.0001166797875002E-2</v>
@@ -7114,7 +7108,7 @@
         <v>93</v>
       </c>
       <c r="M130" s="13">
-        <v>41516</v>
+        <v>41217</v>
       </c>
       <c r="O130" s="8">
         <v>5.8058200810457102E-2</v>
@@ -7161,7 +7155,7 @@
         <v>93.3</v>
       </c>
       <c r="M131" s="13">
-        <v>41562</v>
+        <v>41228</v>
       </c>
       <c r="O131" s="8">
         <v>1.31109526893063E-2</v>
@@ -7208,7 +7202,7 @@
         <v>93.8</v>
       </c>
       <c r="M132" s="13">
-        <v>41582</v>
+        <v>41271</v>
       </c>
       <c r="O132" s="8">
         <v>3.3187639431439202E-2</v>
@@ -7255,7 +7249,7 @@
         <v>95.8</v>
       </c>
       <c r="M133" s="13">
-        <v>41400</v>
+        <v>41307</v>
       </c>
       <c r="O133" s="8">
         <v>2.33420962618727E-2</v>
@@ -7302,7 +7296,7 @@
         <v>98.3</v>
       </c>
       <c r="M134" s="13">
-        <v>40979</v>
+        <v>41330</v>
       </c>
       <c r="O134" s="8">
         <v>2.7157426752474099E-2</v>
@@ -7349,7 +7343,7 @@
         <v>98.9</v>
       </c>
       <c r="M135" s="13">
-        <v>41020</v>
+        <v>41382</v>
       </c>
       <c r="O135" s="8">
         <v>-3.22810954099957E-2</v>
@@ -7396,7 +7390,7 @@
         <v>101.8</v>
       </c>
       <c r="M136" s="13">
-        <v>41116</v>
+        <v>41421</v>
       </c>
       <c r="O136" s="8">
         <v>6.5034918411234002E-2</v>
@@ -7443,7 +7437,7 @@
         <v>103.1</v>
       </c>
       <c r="M137" s="13">
-        <v>41312</v>
+        <v>41466</v>
       </c>
       <c r="O137" s="8">
         <v>-2.9819576373086E-2</v>
@@ -7490,7 +7484,7 @@
         <v>102.4</v>
       </c>
       <c r="M138" s="13">
-        <v>41497</v>
+        <v>41512</v>
       </c>
       <c r="O138" s="8">
         <v>1.1254472695887001E-2</v>
@@ -7537,7 +7531,7 @@
         <v>102</v>
       </c>
       <c r="M139" s="13">
-        <v>41603</v>
+        <v>41567</v>
       </c>
       <c r="O139" s="8">
         <v>-2.9925874226060901E-2</v>
@@ -7584,7 +7578,7 @@
         <v>102.6</v>
       </c>
       <c r="M140" s="13">
-        <v>41617</v>
+        <v>41573</v>
       </c>
       <c r="O140" s="8">
         <v>-0.21309573317035399</v>
@@ -7631,7 +7625,7 @@
         <v>101.8</v>
       </c>
       <c r="M141" s="13">
-        <v>41737</v>
+        <v>41645</v>
       </c>
       <c r="O141" s="8">
         <v>-5.0127146976390001E-2</v>
@@ -7678,7 +7672,7 @@
         <v>103.4</v>
       </c>
       <c r="M142" s="13">
-        <v>41968</v>
+        <v>41684</v>
       </c>
       <c r="O142" s="8">
         <v>0.109927632860542</v>
@@ -7725,7 +7719,7 @@
         <v>103.7</v>
       </c>
       <c r="M143" s="13">
-        <v>42033</v>
+        <v>41708</v>
       </c>
       <c r="O143" s="8">
         <v>-8.5853722212210198E-3</v>
@@ -7772,7 +7766,7 @@
         <v>104.2</v>
       </c>
       <c r="M144" s="13">
-        <v>42062</v>
+        <v>41760</v>
       </c>
       <c r="O144" s="8">
         <v>-3.1784894387906E-2</v>
@@ -7819,7 +7813,7 @@
         <v>103.4</v>
       </c>
       <c r="M145" s="13">
-        <v>41899</v>
+        <v>41815</v>
       </c>
       <c r="O145" s="8">
         <v>9.0787929760299604E-2</v>
@@ -7866,7 +7860,7 @@
         <v>105.3</v>
       </c>
       <c r="M146" s="13">
-        <v>41549</v>
+        <v>41896</v>
       </c>
       <c r="O146" s="8">
         <v>5.96752641347056E-2</v>
@@ -7913,7 +7907,7 @@
         <v>106.7</v>
       </c>
       <c r="M147" s="13">
-        <v>41534</v>
+        <v>41896</v>
       </c>
       <c r="O147" s="8">
         <v>1.3149590428955801E-2</v>
@@ -7960,7 +7954,7 @@
         <v>108.3</v>
       </c>
       <c r="M148" s="13">
-        <v>41639</v>
+        <v>41940</v>
       </c>
       <c r="O148" s="8">
         <v>-2.7086550263575801E-2</v>
@@ -8007,7 +8001,7 @@
         <v>108.8</v>
       </c>
       <c r="M149" s="13">
-        <v>41826</v>
+        <v>41973</v>
       </c>
       <c r="O149" s="8">
         <v>-7.6319299145273703E-2</v>
@@ -8054,7 +8048,7 @@
         <v>107.4</v>
       </c>
       <c r="M150" s="13">
-        <v>42020</v>
+        <v>42025</v>
       </c>
       <c r="O150" s="8">
         <v>2.39588747716333E-2</v>
@@ -8101,7 +8095,7 @@
         <v>106.1</v>
       </c>
       <c r="M151" s="13">
-        <v>42097</v>
+        <v>42050</v>
       </c>
       <c r="O151" s="8">
         <v>5.3996345284742703E-2</v>
@@ -8148,7 +8142,7 @@
         <v>107.1</v>
       </c>
       <c r="M152" s="13">
-        <v>42139</v>
+        <v>42085</v>
       </c>
       <c r="O152" s="8">
         <v>2.8893744541173699E-2</v>
@@ -8195,7 +8189,7 @@
         <v>109.3</v>
       </c>
       <c r="M153" s="13">
-        <v>42218</v>
+        <v>42132</v>
       </c>
       <c r="O153" s="8">
         <v>3.4592989299461897E-2</v>
@@ -8242,7 +8236,7 @@
         <v>110.3</v>
       </c>
       <c r="M154" s="13">
-        <v>42398</v>
+        <v>42131</v>
       </c>
       <c r="O154" s="8">
         <v>6.1450296402370003E-3</v>
@@ -8289,7 +8283,7 @@
         <v>109.3</v>
       </c>
       <c r="M155" s="13">
-        <v>42492</v>
+        <v>42174</v>
       </c>
       <c r="O155" s="8">
         <v>1.9756381593703399E-2</v>
@@ -8336,7 +8330,7 @@
         <v>108.1</v>
       </c>
       <c r="M156" s="13">
-        <v>42532</v>
+        <v>42238</v>
       </c>
       <c r="O156" s="8">
         <v>2.7554233588855202E-2</v>
@@ -8383,7 +8377,7 @@
         <v>107.2</v>
       </c>
       <c r="M157" s="13">
-        <v>42338</v>
+        <v>42263</v>
       </c>
       <c r="O157" s="8">
         <v>2.1271271087686099E-2</v>
@@ -8430,7 +8424,7 @@
         <v>109.8</v>
       </c>
       <c r="M158" s="13">
-        <v>41915</v>
+        <v>42259</v>
       </c>
       <c r="O158" s="8">
         <v>-4.4271451052182399E-3</v>
@@ -8477,7 +8471,7 @@
         <v>111.1</v>
       </c>
       <c r="M159" s="13">
-        <v>41939</v>
+        <v>42299</v>
       </c>
       <c r="O159" s="8">
         <v>6.9009513620414999E-3</v>
@@ -8524,7 +8518,7 @@
         <v>109.5</v>
       </c>
       <c r="M160" s="13">
-        <v>41989</v>
+        <v>42280</v>
       </c>
       <c r="O160" s="8">
         <v>1.50744151153557E-2</v>
@@ -8571,7 +8565,7 @@
         <v>110</v>
       </c>
       <c r="M161" s="13">
-        <v>42141</v>
+        <v>42278</v>
       </c>
       <c r="O161" s="8">
         <v>5.3525894907714602E-2</v>
@@ -8618,7 +8612,7 @@
         <v>109.5</v>
       </c>
       <c r="M162" s="13">
-        <v>42328</v>
+        <v>42325</v>
       </c>
       <c r="O162" s="8">
         <v>-4.7791556243044701E-2</v>
@@ -8665,7 +8659,7 @@
         <v>109.4</v>
       </c>
       <c r="M163" s="13">
-        <v>42396</v>
+        <v>42340</v>
       </c>
       <c r="O163" s="8">
         <v>3.90250697989281E-2</v>
@@ -8712,7 +8706,7 @@
         <v>110.6</v>
       </c>
       <c r="M164" s="13">
-        <v>42460</v>
+        <v>42397</v>
       </c>
       <c r="O164" s="8">
         <v>-2.1103238979252498E-2</v>
@@ -8759,7 +8753,7 @@
         <v>110.4</v>
       </c>
       <c r="M165" s="13">
-        <v>42483</v>
+        <v>42407</v>
       </c>
       <c r="O165" s="8">
         <v>5.8858010903346497E-2</v>
@@ -8806,7 +8800,7 @@
         <v>110.8</v>
       </c>
       <c r="M166" s="13">
-        <v>42690</v>
+        <v>42441</v>
       </c>
       <c r="O166" s="8">
         <v>4.9875499288914299E-2</v>
@@ -8853,7 +8847,7 @@
         <v>109.2</v>
       </c>
       <c r="M167" s="13">
-        <v>42804</v>
+        <v>42492</v>
       </c>
       <c r="O167" s="8">
         <v>4.0286966294466701E-2</v>
@@ -8900,7 +8894,7 @@
         <v>108.2</v>
       </c>
       <c r="M168" s="13">
-        <v>42798</v>
+        <v>42513</v>
       </c>
       <c r="O168" s="8">
         <v>1.54939838815942E-2</v>
@@ -8947,7 +8941,7 @@
         <v>108.7</v>
       </c>
       <c r="M169" s="13">
-        <v>42595</v>
+        <v>42527</v>
       </c>
       <c r="O169" s="8">
         <v>-2.6056341199826201E-2</v>
@@ -8994,7 +8988,7 @@
         <v>107.9</v>
       </c>
       <c r="M170" s="13">
-        <v>42273</v>
+        <v>42616</v>
       </c>
       <c r="O170" s="8">
         <v>4.0598083124759703E-2</v>
@@ -9041,7 +9035,7 @@
         <v>108.2</v>
       </c>
       <c r="M171" s="13">
-        <v>42295</v>
+        <v>42650</v>
       </c>
       <c r="O171" s="8">
         <v>-1.4149237607458801E-2</v>
@@ -9088,7 +9082,7 @@
         <v>107.8</v>
       </c>
       <c r="M172" s="13">
-        <v>42397</v>
+        <v>42674</v>
       </c>
       <c r="O172" s="8">
         <v>4.9397214256607898E-3</v>
@@ -9135,7 +9129,7 @@
         <v>108.6</v>
       </c>
       <c r="M173" s="13">
-        <v>42600</v>
+        <v>42729</v>
       </c>
       <c r="O173" s="8">
         <v>3.4796344239657301E-2</v>
@@ -9182,7 +9176,7 @@
         <v>108.6</v>
       </c>
       <c r="M174" s="13">
-        <v>42742</v>
+        <v>42735</v>
       </c>
       <c r="O174" s="8">
         <v>-1.1144666830492899E-2</v>
@@ -9229,7 +9223,7 @@
         <v>109.1</v>
       </c>
       <c r="M175" s="13">
-        <v>42820</v>
+        <v>42759</v>
       </c>
       <c r="O175" s="8">
         <v>-4.4246059091339197E-2</v>
@@ -9276,7 +9270,7 @@
         <v>108.9</v>
       </c>
       <c r="M176" s="13">
-        <v>42867</v>
+        <v>42801</v>
       </c>
       <c r="O176" s="8">
         <v>6.6416828655899698E-3</v>
@@ -9323,7 +9317,7 @@
         <v>108.3</v>
       </c>
       <c r="M177" s="13">
-        <v>42850</v>
+        <v>42786</v>
       </c>
       <c r="O177" s="8">
         <v>4.3599878355316001E-4</v>
@@ -9370,7 +9364,7 @@
         <v>108.4</v>
       </c>
       <c r="M178" s="13">
-        <v>43051</v>
+        <v>42816</v>
       </c>
       <c r="O178" s="8">
         <v>-1.56833548136621E-2</v>
@@ -9417,7 +9411,7 @@
         <v>106.9</v>
       </c>
       <c r="M179" s="13">
-        <v>43161</v>
+        <v>42858</v>
       </c>
       <c r="O179" s="8">
         <v>6.7768723717097898E-2</v>
@@ -9464,7 +9458,7 @@
         <v>105.7</v>
       </c>
       <c r="M180" s="13">
-        <v>43105</v>
+        <v>42828</v>
       </c>
       <c r="O180" s="8">
         <v>-1.7719685913595701E-2</v>
@@ -9511,7 +9505,7 @@
         <v>101.6</v>
       </c>
       <c r="M181" s="13">
-        <v>42910</v>
+        <v>42843</v>
       </c>
       <c r="O181" s="8">
         <v>8.6764256635232698E-2</v>
@@ -9558,7 +9552,7 @@
         <v>98.3</v>
       </c>
       <c r="M182" s="13">
-        <v>42539</v>
+        <v>42876</v>
       </c>
       <c r="O182" s="8">
         <v>6.4046183917533001E-2</v>
@@ -9605,7 +9599,7 @@
         <v>100.4</v>
       </c>
       <c r="M183" s="13">
-        <v>42559</v>
+        <v>42905</v>
       </c>
       <c r="O183" s="8">
         <v>4.8324522718719003E-2</v>
@@ -9652,7 +9646,7 @@
         <v>101.8</v>
       </c>
       <c r="M184" s="13">
-        <v>42717</v>
+        <v>42980</v>
       </c>
       <c r="O184" s="8">
         <v>-4.37113158841669E-2</v>
@@ -9699,7 +9693,7 @@
         <v>102.3</v>
       </c>
       <c r="M185" s="13">
-        <v>42917</v>
+        <v>43036</v>
       </c>
       <c r="O185" s="8">
         <v>-3.54725011116841E-3</v>
@@ -9746,7 +9740,7 @@
         <v>103.3</v>
       </c>
       <c r="M186" s="13">
-        <v>43079</v>
+        <v>43070</v>
       </c>
       <c r="O186" s="8">
         <v>-4.1944964251854303E-2</v>
@@ -9793,7 +9787,7 @@
         <v>102.8</v>
       </c>
       <c r="M187" s="13">
-        <v>43184</v>
+        <v>43120</v>
       </c>
       <c r="O187" s="8">
         <v>3.2718040351463501E-2</v>
@@ -9840,7 +9834,7 @@
         <v>102.3</v>
       </c>
       <c r="M188" s="13">
-        <v>43240</v>
+        <v>43177</v>
       </c>
       <c r="O188" s="8">
         <v>-9.7397802390855007E-2</v>
@@ -9887,7 +9881,7 @@
         <v>100.2</v>
       </c>
       <c r="M189" s="13">
-        <v>43262</v>
+        <v>43209</v>
       </c>
       <c r="O189" s="8">
         <v>-6.0160962650682499E-2</v>
@@ -9934,7 +9928,7 @@
         <v>98.4</v>
       </c>
       <c r="M190" s="13">
-        <v>43472</v>
+        <v>43249</v>
       </c>
       <c r="O190" s="8">
         <v>0.116138710406931</v>
@@ -9981,7 +9975,7 @@
         <v>97.6</v>
       </c>
       <c r="M191" s="13">
-        <v>43589</v>
+        <v>43296</v>
       </c>
       <c r="O191" s="8">
         <v>4.7875457776937601E-2</v>
@@ -10028,7 +10022,7 @@
         <v>97.7</v>
       </c>
       <c r="M192" s="13">
-        <v>43623</v>
+        <v>43351</v>
       </c>
       <c r="O192" s="8">
         <v>-5.7798119798164301E-2</v>
@@ -10075,7 +10069,7 @@
         <v>95</v>
       </c>
       <c r="M193" s="13">
-        <v>43465</v>
+        <v>43394</v>
       </c>
       <c r="O193" s="8">
         <v>-9.2065742891163496E-2</v>
@@ -10122,7 +10116,7 @@
         <v>92.7</v>
       </c>
       <c r="M194" s="13">
-        <v>43064</v>
+        <v>43391</v>
       </c>
       <c r="O194" s="8">
         <v>-3.1382033864236498E-2</v>
@@ -10169,7 +10163,7 @@
         <v>91.8</v>
       </c>
       <c r="M195" s="13">
-        <v>43120</v>
+        <v>43457</v>
       </c>
       <c r="O195" s="8">
         <v>4.8322596012733102E-2</v>
@@ -10216,7 +10210,7 @@
         <v>92.7</v>
       </c>
       <c r="M196" s="13">
-        <v>43271</v>
+        <v>43522</v>
       </c>
       <c r="O196" s="8">
         <v>7.3443841583866699E-3</v>
@@ -10263,7 +10257,7 @@
         <v>93.6</v>
       </c>
       <c r="M197" s="13">
-        <v>43445</v>
+        <v>43557</v>
       </c>
       <c r="O197" s="8">
         <v>2.2045391335192101E-2</v>
@@ -10310,7 +10304,7 @@
         <v>95</v>
       </c>
       <c r="M198" s="13">
-        <v>43622</v>
+        <v>43614</v>
       </c>
       <c r="O198" s="8">
         <v>-5.8448700832512301E-2</v>
@@ -10357,7 +10351,7 @@
         <v>96.2</v>
       </c>
       <c r="M199" s="13">
-        <v>43735</v>
+        <v>43674</v>
       </c>
       <c r="O199" s="8">
         <v>6.5706877725263596E-2</v>
@@ -10404,7 +10398,7 @@
         <v>95.1</v>
       </c>
       <c r="M200" s="13">
-        <v>43733</v>
+        <v>43679</v>
       </c>
       <c r="O200" s="8">
         <v>2.4386120792158301E-2</v>
@@ -10451,7 +10445,7 @@
         <v>94.3</v>
       </c>
       <c r="M201" s="13">
-        <v>43801</v>
+        <v>43759</v>
       </c>
       <c r="O201" s="8">
         <v>-7.7399951300858296E-3</v>
@@ -10498,7 +10492,7 @@
         <v>94.9</v>
       </c>
       <c r="M202" s="13">
-        <v>44040</v>
+        <v>43829</v>
       </c>
       <c r="O202" s="8">
         <v>1.4544081581430401E-2</v>
@@ -10545,7 +10539,7 @@
         <v>96.2</v>
       </c>
       <c r="M203" s="13">
-        <v>44149</v>
+        <v>43868</v>
       </c>
       <c r="O203" s="8">
         <v>-2.3196069444981799E-3</v>
@@ -10592,7 +10586,7 @@
         <v>95.2</v>
       </c>
       <c r="M204" s="13">
-        <v>44193</v>
+        <v>43924</v>
       </c>
       <c r="O204" s="8">
         <v>7.6050023049042195E-2</v>
@@ -10639,7 +10633,7 @@
         <v>97.3</v>
       </c>
       <c r="M205" s="13">
-        <v>44060</v>
+        <v>43981</v>
       </c>
       <c r="O205" s="8">
         <v>4.7140450460680904E-3</v>
@@ -10686,7 +10680,7 @@
         <v>98.2</v>
       </c>
       <c r="M206" s="13">
-        <v>43689</v>
+        <v>43997</v>
       </c>
       <c r="O206" s="8">
         <v>2.55986740488847E-2</v>
@@ -10733,7 +10727,7 @@
         <v>98.4</v>
       </c>
       <c r="M207" s="13">
-        <v>43727</v>
+        <v>44045</v>
       </c>
       <c r="O207" s="8">
         <v>3.9633663532784497E-2</v>
@@ -10780,7 +10774,7 @@
         <v>97.5</v>
       </c>
       <c r="M208" s="13">
-        <v>43876</v>
+        <v>44119</v>
       </c>
       <c r="O208" s="8">
         <v>1.0112021500111401E-2</v>
@@ -10827,7 +10821,7 @@
         <v>98.3</v>
       </c>
       <c r="M209" s="13">
-        <v>44050</v>
+        <v>44162</v>
       </c>
       <c r="O209" s="8">
         <v>1.41342164371014E-2</v>
@@ -10874,7 +10868,7 @@
         <v>96.9</v>
       </c>
       <c r="M210" s="13">
-        <v>44215</v>
+        <v>44210</v>
       </c>
       <c r="O210" s="8">
         <v>-2.3251838565112599E-2</v>
@@ -10921,7 +10915,7 @@
         <v>96.1</v>
       </c>
       <c r="M211" s="13">
-        <v>44337</v>
+        <v>44284</v>
       </c>
       <c r="O211" s="8">
         <v>-1.6926884920629E-2</v>
@@ -10968,7 +10962,7 @@
         <v>95.9</v>
       </c>
       <c r="M212" s="13">
-        <v>44376</v>
+        <v>44336</v>
       </c>
       <c r="O212" s="8">
         <v>-5.1634039015926404E-3</v>
@@ -11015,7 +11009,7 @@
         <v>96.3</v>
       </c>
       <c r="M213" s="13">
-        <v>44411</v>
+        <v>44379</v>
       </c>
       <c r="O213" s="8">
         <v>6.21481709604765E-2</v>
@@ -11062,7 +11056,7 @@
         <v>97.5</v>
       </c>
       <c r="M214" s="13">
-        <v>44626</v>
+        <v>44423</v>
       </c>
       <c r="O214" s="8">
         <v>3.0757151494398699E-2</v>
@@ -11109,7 +11103,7 @@
         <v>97.4</v>
       </c>
       <c r="M215" s="13">
-        <v>44725</v>
+        <v>44451</v>
       </c>
       <c r="O215" s="8">
         <v>-1.5662189706576499E-2</v>
@@ -11156,7 +11150,7 @@
         <v>98.7</v>
       </c>
       <c r="M216" s="13">
-        <v>44784</v>
+        <v>44515</v>
       </c>
       <c r="O216" s="8">
         <v>-8.1985177085393008E-3</v>
@@ -11203,7 +11197,7 @@
         <v>98.5</v>
       </c>
       <c r="M217" s="13">
-        <v>44663</v>
+        <v>44573</v>
       </c>
       <c r="O217" s="8">
         <v>2.0825785770625799E-2</v>
@@ -11250,7 +11244,7 @@
         <v>98.9</v>
       </c>
       <c r="M218" s="13">
-        <v>44371</v>
+        <v>44659</v>
       </c>
       <c r="O218" s="8">
         <v>-5.8836178729487501E-2</v>
@@ -11297,7 +11291,7 @@
         <v>98.5</v>
       </c>
       <c r="M219" s="13">
-        <v>44388</v>
+        <v>44686</v>
       </c>
       <c r="O219" s="8">
         <v>-2.76481920609708E-2</v>
@@ -11344,7 +11338,7 @@
         <v>97.9</v>
       </c>
       <c r="M220" s="13">
-        <v>44493</v>
+        <v>44730</v>
       </c>
       <c r="O220" s="8">
         <v>4.1722284476579198E-2</v>
@@ -11391,7 +11385,7 @@
         <v>99.5</v>
       </c>
       <c r="M221" s="13">
-        <v>44669</v>
+        <v>44784</v>
       </c>
       <c r="O221" s="8">
         <v>-5.7268535689125599E-4</v>
@@ -11438,7 +11432,7 @@
         <v>101.9</v>
       </c>
       <c r="M222" s="13">
-        <v>44842</v>
+        <v>44847</v>
       </c>
       <c r="O222" s="8">
         <v>-2.3997857696789599E-2</v>
@@ -11485,7 +11479,7 @@
         <v>102.4</v>
       </c>
       <c r="M223" s="13">
-        <v>44912</v>
+        <v>44871</v>
       </c>
       <c r="O223" s="8">
         <v>3.9787817818036003E-2</v>
@@ -11532,7 +11526,7 @@
         <v>102.3</v>
       </c>
       <c r="M224" s="13">
-        <v>44942</v>
+        <v>44913</v>
       </c>
       <c r="O224" s="8">
         <v>-3.5080923832737199E-2</v>
@@ -11579,7 +11573,7 @@
         <v>103.1</v>
       </c>
       <c r="M225" s="13">
-        <v>44986</v>
+        <v>44963</v>
       </c>
       <c r="O225" s="8">
         <v>-9.5348414473441796E-3</v>
@@ -11626,7 +11620,7 @@
         <v>105.1</v>
       </c>
       <c r="M226" s="13">
-        <v>45159</v>
+        <v>44962</v>
       </c>
       <c r="O226" s="8">
         <v>-6.7486782228227696E-2</v>
@@ -11673,7 +11667,7 @@
         <v>106.1</v>
       </c>
       <c r="M227" s="13">
-        <v>45271</v>
+        <v>45002</v>
       </c>
       <c r="O227" s="8">
         <v>-1.67607205951796E-2</v>
@@ -11720,7 +11714,7 @@
         <v>108</v>
       </c>
       <c r="M228" s="13">
-        <v>45323</v>
+        <v>45056</v>
       </c>
       <c r="O228" s="8">
         <v>-6.4036713152630001E-2</v>
@@ -11767,7 +11761,7 @@
         <v>103.5</v>
       </c>
       <c r="M229" s="13">
-        <v>45183</v>
+        <v>45087</v>
       </c>
       <c r="O229" s="8">
         <v>5.6534283831409099E-2</v>
@@ -11814,7 +11808,7 @@
         <v>101.5</v>
       </c>
       <c r="M230" s="13">
-        <v>44866</v>
+        <v>45131</v>
       </c>
       <c r="O230" s="8">
         <v>3.0197012166079101E-2</v>
@@ -11861,7 +11855,7 @@
         <v>101.7</v>
       </c>
       <c r="M231" s="13">
-        <v>44894</v>
+        <v>45170</v>
       </c>
       <c r="O231" s="8">
         <v>9.0274593453010298E-4</v>
@@ -11908,7 +11902,7 @@
         <v>102.4</v>
       </c>
       <c r="M232" s="13">
-        <v>44983</v>
+        <v>45213</v>
       </c>
       <c r="O232" s="8">
         <v>6.85677754379697E-2</v>
@@ -11955,7 +11949,7 @@
         <v>104.4</v>
       </c>
       <c r="M233" s="13">
-        <v>45150</v>
+        <v>45270</v>
       </c>
       <c r="O233" s="8">
         <v>-5.1296383916635997E-2</v>
@@ -12002,7 +11996,7 @@
         <v>106.1</v>
       </c>
       <c r="M234" s="13">
-        <v>45273</v>
+        <v>45288</v>
       </c>
       <c r="O234" s="8">
         <v>5.57194596484187E-2</v>
@@ -12049,7 +12043,7 @@
         <v>104.9</v>
       </c>
       <c r="M235" s="13">
-        <v>45314</v>
+        <v>45285</v>
       </c>
       <c r="O235" s="8">
         <v>-1.70624874615601E-2</v>
@@ -12096,7 +12090,7 @@
         <v>104.7</v>
       </c>
       <c r="M236" s="13">
-        <v>45333</v>
+        <v>45317</v>
       </c>
       <c r="O236" s="8">
         <v>-2.0703362979372E-2</v>
@@ -12143,7 +12137,7 @@
         <v>103.8</v>
       </c>
       <c r="M237" s="13">
-        <v>45328</v>
+        <v>45313</v>
       </c>
       <c r="O237" s="8">
         <v>4.0124607332764101E-2</v>
@@ -12190,7 +12184,7 @@
         <v>103.8</v>
       </c>
       <c r="M238" s="13">
-        <v>45529</v>
+        <v>45335</v>
       </c>
       <c r="O238" s="8">
         <v>3.4691141411061097E-2</v>
@@ -12237,7 +12231,7 @@
         <v>103.8</v>
       </c>
       <c r="M239" s="13">
-        <v>45639</v>
+        <v>45368</v>
       </c>
       <c r="O239" s="8">
         <v>2.8319514088868999E-2</v>
@@ -12284,7 +12278,7 @@
         <v>103.7</v>
       </c>
       <c r="M240" s="13">
-        <v>45667</v>
+        <v>45403</v>
       </c>
       <c r="O240" s="8">
         <v>9.5372459589704295E-4</v>
@@ -12331,7 +12325,7 @@
         <v>103.6</v>
       </c>
       <c r="M241" s="13">
-        <v>45518</v>
+        <v>45418</v>
       </c>
       <c r="O241" s="8">
         <v>-2.03613643159084E-2</v>
@@ -12378,7 +12372,7 @@
         <v>104.9</v>
       </c>
       <c r="M242" s="13">
-        <v>45205</v>
+        <v>45455</v>
       </c>
       <c r="O242" s="8">
         <v>-8.7834336735301805E-2</v>
@@ -12425,7 +12419,7 @@
         <v>103.9</v>
       </c>
       <c r="M243" s="13">
-        <v>45206</v>
+        <v>45466</v>
       </c>
       <c r="O243" s="8">
         <v>-0.17957870764244499</v>
@@ -12472,7 +12466,7 @@
         <v>101.6</v>
       </c>
       <c r="M244" s="13">
-        <v>45125</v>
+        <v>45344</v>
       </c>
       <c r="O244" s="8">
         <v>8.9088877352494905E-2</v>
@@ -12519,7 +12513,7 @@
         <v>98.6</v>
       </c>
       <c r="M245" s="13">
-        <v>44867</v>
+        <v>44985</v>
       </c>
       <c r="O245" s="8">
         <v>6.4633517047441899E-2</v>
@@ -12566,7 +12560,7 @@
         <v>97.4</v>
       </c>
       <c r="M246" s="13">
-        <v>44726</v>
+        <v>44750</v>
       </c>
       <c r="O246" s="8">
         <v>6.0616659617544102E-2</v>
@@ -12613,7 +12607,7 @@
         <v>98.7</v>
       </c>
       <c r="M247" s="13">
-        <v>44739</v>
+        <v>44716</v>
       </c>
       <c r="O247" s="8">
         <v>1.97420032540307E-4</v>
@@ -12660,7 +12654,7 @@
         <v>98</v>
       </c>
       <c r="M248" s="13">
-        <v>44748</v>
+        <v>44740</v>
       </c>
       <c r="O248" s="8">
         <v>5.0054078357490497E-2</v>
@@ -12707,7 +12701,7 @@
         <v>97.6</v>
       </c>
       <c r="M249" s="13">
-        <v>44780</v>
+        <v>44774</v>
       </c>
       <c r="O249" s="8">
         <v>-1.43664356381485E-2</v>
@@ -12754,7 +12748,7 @@
         <v>96.9</v>
       </c>
       <c r="M250" s="13">
-        <v>45018</v>
+        <v>44832</v>
       </c>
       <c r="O250" s="8">
         <v>-9.9126163878370505E-2</v>
@@ -12801,7 +12795,7 @@
         <v>97</v>
       </c>
       <c r="M251" s="13">
-        <v>45136</v>
+        <v>44871</v>
       </c>
       <c r="O251" s="8">
         <v>0.13985280517704099</v>
@@ -12848,7 +12842,7 @@
         <v>96</v>
       </c>
       <c r="M252" s="13">
-        <v>45090</v>
+        <v>44835</v>
       </c>
       <c r="O252" s="8">
         <v>3.1666552648804497E-2</v>
@@ -12895,7 +12889,7 @@
         <v>97.4</v>
       </c>
       <c r="M253" s="13">
-        <v>44945</v>
+        <v>44846</v>
       </c>
       <c r="O253" s="8">
         <v>-2.1061019894339901E-2</v>
@@ -12942,7 +12936,7 @@
         <v>102.6</v>
       </c>
       <c r="M254" s="13">
-        <v>44573</v>
+        <v>44811</v>
       </c>
       <c r="O254" s="8">
         <v>2.5969925810608498E-2</v>
@@ -12989,7 +12983,7 @@
         <v>104.1</v>
       </c>
       <c r="M255" s="13">
-        <v>44552</v>
+        <v>44795</v>
       </c>
       <c r="O255" s="8">
         <v>8.4931413271505093E-2</v>
@@ -13036,7 +13030,7 @@
         <v>106.2</v>
       </c>
       <c r="M256" s="13">
-        <v>44642</v>
+        <v>44847</v>
       </c>
       <c r="O256" s="8">
         <v>8.4640403455811305E-3</v>
@@ -13083,7 +13077,7 @@
         <v>106.1</v>
       </c>
       <c r="M257" s="13">
-        <v>44754</v>
+        <v>44870</v>
       </c>
       <c r="O257" s="8">
         <v>1.8668562777554201E-2</v>
@@ -13130,7 +13124,7 @@
         <v>106.7</v>
       </c>
       <c r="M258" s="13">
-        <v>44865</v>
+        <v>44890</v>
       </c>
       <c r="O258" s="8">
         <v>7.1019652901185299E-3</v>
@@ -13177,7 +13171,7 @@
         <v>107.6</v>
       </c>
       <c r="M259" s="13">
-        <v>45026</v>
+        <v>45003</v>
       </c>
       <c r="O259" s="8">
         <v>8.5917461676032801E-4</v>
@@ -13224,7 +13218,7 @@
         <v>109</v>
       </c>
       <c r="M260" s="13">
-        <v>45082</v>
+        <v>45083</v>
       </c>
       <c r="O260" s="8">
         <v>1.8528574508760401E-2</v>
@@ -13271,7 +13265,7 @@
         <v>109.4</v>
       </c>
       <c r="M261" s="13">
-        <v>45143</v>
+        <v>45146</v>
       </c>
       <c r="O261" s="8">
         <v>-3.6948084477158402E-2</v>
@@ -13318,7 +13312,7 @@
         <v>110.1</v>
       </c>
       <c r="M262" s="13">
-        <v>45375</v>
+        <v>45194</v>
       </c>
       <c r="O262" s="8">
         <v>2.7664870670250301E-2</v>
@@ -13365,7 +13359,7 @@
         <v>114.6</v>
       </c>
       <c r="M263" s="13">
-        <v>45489</v>
+        <v>45224</v>
       </c>
       <c r="O263" s="8">
         <v>-3.8241794617819701E-2</v>
@@ -13412,7 +13406,7 @@
         <v>116.7</v>
       </c>
       <c r="M264" s="13">
-        <v>45542</v>
+        <v>45289</v>
       </c>
       <c r="O264" s="8">
         <v>5.0663131173992702E-2</v>
@@ -13459,7 +13453,7 @@
         <v>115</v>
       </c>
       <c r="M265" s="13">
-        <v>45447</v>
+        <v>45345</v>
       </c>
       <c r="O265" s="8">
         <v>-2.6386232778426302E-2</v>
@@ -13506,7 +13500,7 @@
         <v>123.7</v>
       </c>
       <c r="M266" s="13">
-        <v>45187</v>
+        <v>45429</v>
       </c>
       <c r="O266" s="8">
         <v>-6.7523522443023495E-2</v>
@@ -13553,7 +13547,7 @@
         <v>127.4</v>
       </c>
       <c r="M267" s="13">
-        <v>45229</v>
+        <v>45472</v>
       </c>
       <c r="O267" s="8">
         <v>-3.2047333526570299E-3</v>
@@ -13600,7 +13594,7 @@
         <v>146.1</v>
       </c>
       <c r="M268" s="13">
-        <v>45332</v>
+        <v>45527</v>
       </c>
       <c r="O268" s="8">
         <v>-2.22275647371468E-2</v>
@@ -13647,7 +13641,7 @@
         <v>142.69999999999999</v>
       </c>
       <c r="M269" s="13">
-        <v>45448</v>
+        <v>45558</v>
       </c>
       <c r="O269" s="8">
         <v>2.0394401058499802E-2</v>
@@ -13694,7 +13688,7 @@
         <v>146.69999999999999</v>
       </c>
       <c r="M270" s="13">
-        <v>45577</v>
+        <v>45599</v>
       </c>
       <c r="O270" s="8">
         <v>-0.118242463260449</v>
@@ -13741,7 +13735,7 @@
         <v>147.80000000000001</v>
       </c>
       <c r="M271" s="13">
-        <v>45658</v>
+        <v>45628</v>
       </c>
       <c r="O271" s="8">
         <v>5.3331130023282797E-2</v>
@@ -13788,7 +13782,7 @@
         <v>147.80000000000001</v>
       </c>
       <c r="M272" s="13">
-        <v>45614</v>
+        <v>45616</v>
       </c>
       <c r="O272" s="8">
         <v>-4.9334796182296997E-2</v>
@@ -13835,7 +13829,7 @@
         <v>148.6</v>
       </c>
       <c r="M273" s="13">
-        <v>45665</v>
+        <v>45676</v>
       </c>
       <c r="O273" s="8">
         <v>-5.7781139976897898E-2</v>
@@ -13882,7 +13876,7 @@
         <v>158.80000000000001</v>
       </c>
       <c r="M274" s="13">
-        <v>45896</v>
+        <v>45723</v>
       </c>
       <c r="O274" s="8">
         <v>8.9888239618305804E-2</v>
@@ -13929,7 +13923,7 @@
         <v>164.5</v>
       </c>
       <c r="M275" s="13">
-        <v>46017</v>
+        <v>45757</v>
       </c>
       <c r="O275" s="8">
         <v>8.2742838172361402E-2</v>
@@ -13976,7 +13970,7 @@
         <v>163.5</v>
       </c>
       <c r="M276" s="13">
-        <v>46023</v>
+        <v>45773</v>
       </c>
       <c r="O276" s="8">
         <v>-3.3438119878111301E-2</v>
@@ -14023,7 +14017,7 @@
         <v>143.9</v>
       </c>
       <c r="M277" s="13">
-        <v>45901</v>
+        <v>45799</v>
       </c>
       <c r="O277" s="8">
         <v>8.2980635179399798E-2</v>
@@ -14070,7 +14064,7 @@
         <v>154.80000000000001</v>
       </c>
       <c r="M278" s="13">
-        <v>45599</v>
+        <v>45846</v>
       </c>
       <c r="O278" s="8">
         <v>1.55361363662418E-2</v>
@@ -14117,7 +14111,7 @@
         <v>154.9</v>
       </c>
       <c r="M279" s="13">
-        <v>45642</v>
+        <v>45885</v>
       </c>
       <c r="O279" s="8">
         <v>1.7016631153158102E-2</v>
@@ -14164,7 +14158,7 @@
         <v>155</v>
       </c>
       <c r="M280" s="13">
-        <v>45731</v>
+        <v>45917</v>
       </c>
       <c r="O280" s="8">
         <v>1.8607743939233101E-2</v>
@@ -14211,7 +14205,7 @@
         <v>156.1</v>
       </c>
       <c r="M281" s="13">
-        <v>45825</v>
+        <v>45925</v>
       </c>
       <c r="O281" s="8">
         <v>-1.6359326694969301E-2</v>
@@ -14258,7 +14252,7 @@
         <v>154</v>
       </c>
       <c r="M282" s="13">
-        <v>45928</v>
+        <v>45940</v>
       </c>
       <c r="O282" s="8">
         <v>3.04237017694611E-2</v>
@@ -14305,7 +14299,7 @@
         <v>153.69999999999999</v>
       </c>
       <c r="M283" s="13">
-        <v>45992</v>
+        <v>45955</v>
       </c>
       <c r="O283" s="8">
         <v>1.8342723779730001E-2</v>
@@ -14352,7 +14346,7 @@
         <v>153.6</v>
       </c>
       <c r="M284" s="13">
-        <v>45955</v>
+        <v>45959</v>
       </c>
       <c r="O284" s="8">
         <v>-3.0857012954521999E-2</v>
@@ -14399,7 +14393,7 @@
         <v>156.5</v>
       </c>
       <c r="M285" s="13">
-        <v>45932</v>
+        <v>45951</v>
       </c>
       <c r="O285" s="8">
         <v>-3.5780039258788997E-2</v>
@@ -14446,7 +14440,7 @@
         <v>157.6</v>
       </c>
       <c r="M286" s="13">
-        <v>46108</v>
+        <v>45946</v>
       </c>
       <c r="O286" s="8">
         <v>-3.8170131083722601E-2</v>
@@ -14493,7 +14487,7 @@
         <v>154.69999999999999</v>
       </c>
       <c r="M287" s="13">
-        <v>46201</v>
+        <v>45949</v>
       </c>
       <c r="O287" s="8">
         <v>9.0637663864162804E-2</v>
@@ -14540,7 +14534,7 @@
         <v>151.6</v>
       </c>
       <c r="M288" s="13">
-        <v>46218</v>
+        <v>45972</v>
       </c>
       <c r="O288" s="8">
         <v>3.2532962444236098E-2</v>
@@ -14587,7 +14581,7 @@
         <v>148.4</v>
       </c>
       <c r="M289" s="13">
-        <v>46089</v>
+        <v>45988</v>
       </c>
       <c r="O289" s="8">
         <v>9.0398672890046293E-3</v>
@@ -14634,7 +14628,7 @@
         <v>150.19999999999999</v>
       </c>
       <c r="M290" s="13">
-        <v>45718</v>
+        <v>45970</v>
       </c>
       <c r="O290" s="8">
         <v>4.4795576943434098E-2</v>
@@ -14681,7 +14675,7 @@
         <v>150.9</v>
       </c>
       <c r="M291" s="13">
-        <v>45732</v>
+        <v>45975</v>
       </c>
       <c r="O291" s="8">
         <v>4.5033070925896403E-2</v>
@@ -14728,7 +14722,7 @@
         <v>150.5</v>
       </c>
       <c r="M292" s="13">
-        <v>45807</v>
+        <v>45985</v>
       </c>
       <c r="O292" s="8">
         <v>-3.0768414243720298E-2</v>
@@ -14775,7 +14769,7 @@
         <v>154</v>
       </c>
       <c r="M293" s="13">
-        <v>45903</v>
+        <v>45993</v>
       </c>
       <c r="O293" s="8">
         <v>3.1063042818486201E-2</v>
@@ -14822,7 +14816,7 @@
         <v>152.1</v>
       </c>
       <c r="M294" s="13">
-        <v>46007</v>
+        <v>46009</v>
       </c>
       <c r="O294" s="8">
         <v>-1.42918860376433E-2</v>
@@ -14869,7 +14863,7 @@
         <v>150.30000000000001</v>
       </c>
       <c r="M295" s="13">
-        <v>46029</v>
+        <v>45987</v>
       </c>
       <c r="O295" s="8">
         <v>1.4870752550031299E-2</v>
@@ -14916,7 +14910,7 @@
         <v>150.69999999999999</v>
       </c>
       <c r="M296" s="13">
-        <v>45988</v>
+        <v>45989</v>
       </c>
       <c r="O296" s="8">
         <v>2.12897770064568E-2</v>
@@ -14963,7 +14957,7 @@
         <v>148.5</v>
       </c>
       <c r="M297" s="13">
-        <v>45951</v>
+        <v>45976</v>
       </c>
       <c r="O297" s="8">
         <v>2.1867967557486899E-2</v>
@@ -15010,7 +15004,7 @@
         <v>145.80000000000001</v>
       </c>
       <c r="M298" s="13">
-        <v>46122</v>
+        <v>45971</v>
       </c>
       <c r="O298" s="8">
         <v>-1.28842782964522E-2</v>
@@ -15057,7 +15051,7 @@
         <v>146.4</v>
       </c>
       <c r="M299" s="13">
-        <v>46229</v>
+        <v>45985</v>
       </c>
       <c r="O299" s="8">
         <v>2.83664287347438E-2</v>
@@ -15104,7 +15098,7 @@
         <v>146.1</v>
       </c>
       <c r="M300" s="13">
-        <v>46243</v>
+        <v>45999</v>
       </c>
       <c r="O300" s="8">
         <v>1.43008476777062E-2</v>
@@ -15151,7 +15145,7 @@
         <v>146.19999999999999</v>
       </c>
       <c r="M301" s="13">
-        <v>46111</v>
+        <v>46010</v>
       </c>
       <c r="O301" s="8">
         <v>8.76092112293545E-2</v>
@@ -15198,7 +15192,7 @@
         <v>148.19999999999999</v>
       </c>
       <c r="M302" s="13">
-        <v>45754</v>
+        <v>46008</v>
       </c>
       <c r="O302" s="8">
         <v>3.7010299324510498E-2</v>
@@ -15245,7 +15239,7 @@
         <v>148.9</v>
       </c>
       <c r="M303" s="13">
-        <v>45781</v>
+        <v>46021</v>
       </c>
       <c r="O303" s="8">
         <v>-1.7352113686762E-2</v>
@@ -15292,7 +15286,7 @@
         <v>146.6</v>
       </c>
       <c r="M304" s="13">
-        <v>45841</v>
+        <v>46016</v>
       </c>
       <c r="O304" s="8">
         <v>1.4934747787439299E-2</v>
@@ -15339,7 +15333,7 @@
         <v>145.80000000000001</v>
       </c>
       <c r="M305" s="13">
-        <v>45941</v>
+        <v>46024</v>
       </c>
       <c r="O305" s="8">
         <v>6.4567745552686504E-2</v>
@@ -15386,7 +15380,7 @@
         <v>145.19999999999999</v>
       </c>
       <c r="M306" s="13">
-        <v>46008</v>
+        <v>46002</v>
       </c>
       <c r="O306" s="8">
         <v>-3.6684003381495201E-3</v>
@@ -15433,7 +15427,7 @@
         <v>145.1</v>
       </c>
       <c r="M307" s="13">
-        <v>46036</v>
+        <v>45992</v>
       </c>
       <c r="O307" s="8">
         <v>6.4976181897140597E-3</v>
@@ -15480,7 +15474,7 @@
         <v>145.6</v>
       </c>
       <c r="M308" s="13">
-        <v>45985</v>
+        <v>45984</v>
       </c>
       <c r="O308" s="8">
         <v>-6.80709971585891E-3</v>
@@ -15527,7 +15521,7 @@
         <v>145.1</v>
       </c>
       <c r="M309" s="13">
-        <v>45932</v>
+        <v>45962</v>
       </c>
       <c r="O309" s="8">
         <v>-8.9949423721336096E-4</v>
@@ -15574,7 +15568,7 @@
         <v>144.80000000000001</v>
       </c>
       <c r="M310" s="13">
-        <v>46095</v>
+        <v>45952</v>
       </c>
       <c r="O310" s="8">
         <v>3.2433834859766399E-3</v>
@@ -15621,7 +15615,7 @@
         <v>145.1</v>
       </c>
       <c r="M311" s="13">
-        <v>46188</v>
+        <v>45948</v>
       </c>
       <c r="O311" s="8">
         <v>-5.0847056024565501E-3</v>
@@ -15668,7 +15662,7 @@
         <v>145.9</v>
       </c>
       <c r="M312" s="13">
-        <v>46183</v>
+        <v>45941</v>
       </c>
       <c r="O312" s="8">
         <v>2.7051472580767601E-2</v>
@@ -15715,7 +15709,7 @@
         <v>144.30000000000001</v>
       </c>
       <c r="M313" s="13">
-        <v>46037</v>
+        <v>45935</v>
       </c>
       <c r="O313" s="8">
         <v>2.5679690612724598E-2</v>

</xml_diff>